<commit_message>
Update: dados sellout e kpis
</commit_message>
<xml_diff>
--- a/app/etl/Segmentos.xlsx
+++ b/app/etl/Segmentos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phillipe.silva\Documents\Nexus\app\etl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{905A943B-C0BD-4E9B-AD0E-3EB2ECFDB6C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F380FC-5E11-4801-9DEE-B3A4C4E7855F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5626,7 +5626,7 @@
   <dimension ref="A1:I490"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="35" bestFit="1" customWidth="1"/>
@@ -8077,7 +8077,7 @@
         <v>38</v>
       </c>
       <c r="E85" t="s">
-        <v>1555</v>
+        <v>11</v>
       </c>
       <c r="F85" t="s">
         <v>55</v>
@@ -8138,7 +8138,7 @@
         <v>1556</v>
       </c>
       <c r="F87" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="G87" t="s">
         <v>16</v>
@@ -8193,7 +8193,7 @@
         <v>38</v>
       </c>
       <c r="E89" t="s">
-        <v>1555</v>
+        <v>11</v>
       </c>
       <c r="F89" t="s">
         <v>39</v>
@@ -8251,7 +8251,7 @@
         <v>38</v>
       </c>
       <c r="E91" t="s">
-        <v>1552</v>
+        <v>11</v>
       </c>
       <c r="F91" t="s">
         <v>39</v>
@@ -8280,7 +8280,7 @@
         <v>38</v>
       </c>
       <c r="E92" t="s">
-        <v>1552</v>
+        <v>11</v>
       </c>
       <c r="F92" t="s">
         <v>39</v>
@@ -8309,7 +8309,7 @@
         <v>38</v>
       </c>
       <c r="E93" t="s">
-        <v>1555</v>
+        <v>11</v>
       </c>
       <c r="F93" t="s">
         <v>55</v>
@@ -8338,7 +8338,7 @@
         <v>38</v>
       </c>
       <c r="E94" t="s">
-        <v>1555</v>
+        <v>11</v>
       </c>
       <c r="F94" t="s">
         <v>55</v>
@@ -8367,7 +8367,7 @@
         <v>38</v>
       </c>
       <c r="E95" t="s">
-        <v>1555</v>
+        <v>11</v>
       </c>
       <c r="F95" t="s">
         <v>55</v>
@@ -8396,7 +8396,7 @@
         <v>38</v>
       </c>
       <c r="E96" t="s">
-        <v>1556</v>
+        <v>11</v>
       </c>
       <c r="F96" t="s">
         <v>39</v>
@@ -8425,7 +8425,7 @@
         <v>38</v>
       </c>
       <c r="E97" t="s">
-        <v>1552</v>
+        <v>11</v>
       </c>
       <c r="F97" t="s">
         <v>16</v>
@@ -8454,7 +8454,7 @@
         <v>38</v>
       </c>
       <c r="E98" t="s">
-        <v>1552</v>
+        <v>11</v>
       </c>
       <c r="F98" t="s">
         <v>16</v>
@@ -8483,7 +8483,7 @@
         <v>38</v>
       </c>
       <c r="E99" t="s">
-        <v>1552</v>
+        <v>11</v>
       </c>
       <c r="F99" t="s">
         <v>16</v>
@@ -10249,7 +10249,7 @@
         <v>37</v>
       </c>
       <c r="E160" t="s">
-        <v>1552</v>
+        <v>11</v>
       </c>
       <c r="F160" t="s">
         <v>16</v>
@@ -10452,7 +10452,7 @@
         <v>37</v>
       </c>
       <c r="E167" t="s">
-        <v>1552</v>
+        <v>11</v>
       </c>
       <c r="F167" t="s">
         <v>16</v>
@@ -14222,7 +14222,7 @@
         <v>17</v>
       </c>
       <c r="E297" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F297" t="s">
         <v>11</v>
@@ -14251,7 +14251,7 @@
         <v>13</v>
       </c>
       <c r="E298" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F298" t="s">
         <v>11</v>
@@ -14280,7 +14280,7 @@
         <v>36</v>
       </c>
       <c r="E299" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F299" t="s">
         <v>11</v>
@@ -14309,7 +14309,7 @@
         <v>10</v>
       </c>
       <c r="E300" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F300" t="s">
         <v>11</v>
@@ -14338,7 +14338,7 @@
         <v>18</v>
       </c>
       <c r="E301" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F301" t="s">
         <v>11</v>
@@ -37584,12 +37584,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010077ADB75EDE6CA24D9907F62E3498CFFE" ma:contentTypeVersion="3" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="9e4a933615ec58deeded07da77faa5c5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f6c80a7e-4993-4462-a012-3c1269aac47c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dfd25e57b156fdb3c6d899fc66d2ed42" ns2:_="">
     <xsd:import namespace="f6c80a7e-4993-4462-a012-3c1269aac47c"/>
@@ -37727,6 +37721,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA0CA206-730C-405E-B545-6F223619D12E}">
   <ds:schemaRefs>
@@ -37736,15 +37736,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1F20546-7FB8-473C-993C-8D239BFE1C6F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F883CBD-C14F-4597-A1B4-21AD70EB2EF7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -37760,4 +37751,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1F20546-7FB8-473C-993C-8D239BFE1C6F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fix: Virada de Mês
</commit_message>
<xml_diff>
--- a/app/etl/Segmentos.xlsx
+++ b/app/etl/Segmentos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phillipe.silva\Documents\Nexus\app\etl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F380FC-5E11-4801-9DEE-B3A4C4E7855F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E2D5B89-D05A-48F0-B0DA-D21598ADDD88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4763,7 +4763,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -4787,6 +4787,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5847,7 +5848,7 @@
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E8" t="s">
         <v>11</v>
@@ -8135,7 +8136,7 @@
         <v>38</v>
       </c>
       <c r="E87" t="s">
-        <v>1556</v>
+        <v>11</v>
       </c>
       <c r="F87" t="s">
         <v>11</v>
@@ -8424,7 +8425,7 @@
       <c r="D97" t="s">
         <v>38</v>
       </c>
-      <c r="E97" t="s">
+      <c r="E97" s="9" t="s">
         <v>11</v>
       </c>
       <c r="F97" t="s">
@@ -8453,7 +8454,7 @@
       <c r="D98" t="s">
         <v>38</v>
       </c>
-      <c r="E98" t="s">
+      <c r="E98" s="9" t="s">
         <v>11</v>
       </c>
       <c r="F98" t="s">
@@ -37584,6 +37585,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010077ADB75EDE6CA24D9907F62E3498CFFE" ma:contentTypeVersion="3" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="9e4a933615ec58deeded07da77faa5c5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f6c80a7e-4993-4462-a012-3c1269aac47c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dfd25e57b156fdb3c6d899fc66d2ed42" ns2:_="">
     <xsd:import namespace="f6c80a7e-4993-4462-a012-3c1269aac47c"/>
@@ -37721,12 +37728,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA0CA206-730C-405E-B545-6F223619D12E}">
   <ds:schemaRefs>
@@ -37736,6 +37737,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1F20546-7FB8-473C-993C-8D239BFE1C6F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F883CBD-C14F-4597-A1B4-21AD70EB2EF7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -37751,13 +37761,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1F20546-7FB8-473C-993C-8D239BFE1C6F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>